<commit_message>
Finished 03 general and added 02 chi-square
</commit_message>
<xml_diff>
--- a/Data/FINAL SEAS V1 Dataset.xlsx
+++ b/Data/FINAL SEAS V1 Dataset.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29803"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29721"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{440E658F-504C-4184-A1D3-54AEFF037AE7}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF8869A3-BF46-4A0D-B92A-CF2A23F561F9}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5197" uniqueCount="985">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5198" uniqueCount="985">
   <si>
     <t>subject</t>
   </si>
@@ -3414,7 +3414,17 @@
   <dimension ref="A1:DB112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="2" max="7" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" customWidth="1"/>
+    <col min="9" max="16" width="9.140625" customWidth="1"/>
+    <col min="18" max="27" width="9.140625" customWidth="1"/>
+    <col min="29" max="39" width="9.140625" customWidth="1"/>
+    <col min="41" max="50" width="9.140625" customWidth="1"/>
+    <col min="52" max="62" width="9.140625" customWidth="1"/>
+    <col min="64" max="73" width="9.140625" customWidth="1"/>
+    <col min="75" max="85" width="9.140625" customWidth="1"/>
+    <col min="87" max="96" width="9.140625" customWidth="1"/>
+    <col min="98" max="105" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:106" ht="45.75">
@@ -9265,9 +9275,11 @@
       </c>
       <c r="AA27" s="7"/>
       <c r="AB27" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="AC27" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="AC27" s="7"/>
       <c r="AD27" s="8"/>
       <c r="AE27" s="7"/>
       <c r="AF27" s="8"/>

</xml_diff>